<commit_message>
Apply spreadsheet corrections and green VAT price footer note
Update tarjoukset.xlsx with the corrected product details and replace
the footer's 'oranssi hinta sis. alv.' with 'vihreä hinta sis. alv.'
on both offer pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8Lk915b9RmWmbPNMZUzmb
</commit_message>
<xml_diff>
--- a/viikkotarjoukset/tarjoukset.xlsx
+++ b/viikkotarjoukset/tarjoukset.xlsx
@@ -80,7 +80,7 @@
     <t>Tuore, Suomi, 4kg/kpl</t>
   </si>
   <si>
-    <t>Lagerblad foods lammaspyörykkä 16g</t>
+    <t>Lagerblad Foods lammaspyörykkä 16g</t>
   </si>
   <si>
     <t>Pakaste, Suomi, 6kg/ltk</t>
@@ -104,7 +104,7 @@
     <t>Pangasiusfilee 120-170g</t>
   </si>
   <si>
-    <t>Pakaste, Vietnam, 5kg/ltk</t>
+    <t>Pakaste, Vietnam, 10kg/ltk</t>
   </si>
   <si>
     <t>Merhav Hoki Annospala Luomupaneroitu 50g</t>
@@ -116,7 +116,7 @@
     <t>Familia Pro Porsaan kypsä ulkofileeleike 120g</t>
   </si>
   <si>
-    <t>Pakaste, EU, 7,2kg/ltk</t>
+    <t>Pakaste, Saksa, 7,2kg/ltk</t>
   </si>
   <si>
     <t>HK Uunimakkara 80g</t>
@@ -134,7 +134,7 @@
     <t>Sauvon maustekurkkukuutio</t>
   </si>
   <si>
-    <t>Suomi, 8,2kg. Valutettu paino 4,3kg</t>
+    <t>Suomi, 8,2kg/4.3kg</t>
   </si>
 </sst>
 </file>
@@ -144,7 +144,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -184,6 +184,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -217,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -248,6 +253,9 @@
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
@@ -257,12 +265,15 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -678,7 +689,7 @@
       <c r="F7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="12" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="9" t="s">
@@ -725,7 +736,7 @@
     <row r="9">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="12"/>
+      <c r="C9" s="13"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
@@ -736,7 +747,7 @@
       <c r="B10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="12"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
@@ -770,166 +781,166 @@
       <c r="K12" s="1"/>
     </row>
     <row r="13">
-      <c r="B13" s="13">
+      <c r="B13" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="14">
         <v>46327.0</v>
       </c>
       <c r="D13" s="8">
         <v>5.1</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="15">
         <f t="shared" ref="E13:E18" si="2">D13*1.135</f>
         <v>5.7885</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="16" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="18">
         <v>133952.0</v>
       </c>
-      <c r="K13" s="17"/>
+      <c r="K13" s="19"/>
     </row>
     <row r="14">
-      <c r="B14" s="13">
+      <c r="B14" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="14">
         <v>46327.0</v>
       </c>
       <c r="D14" s="8">
         <v>6.8</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="15">
         <f t="shared" si="2"/>
         <v>7.718</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="G14" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="H14" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="18">
         <v>143955.0</v>
       </c>
-      <c r="K14" s="17"/>
+      <c r="K14" s="19"/>
     </row>
     <row r="15">
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="14">
         <v>46327.0</v>
       </c>
       <c r="D15" s="8">
         <v>8.62</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="15">
         <f t="shared" si="2"/>
         <v>9.7837</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="18">
         <v>129487.0</v>
       </c>
       <c r="K15" s="10"/>
     </row>
     <row r="16">
-      <c r="B16" s="13">
+      <c r="B16" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="14">
         <v>46327.0</v>
       </c>
       <c r="D16" s="8">
         <v>4.75</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="15">
         <f t="shared" si="2"/>
         <v>5.39125</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="18">
         <v>103157.0</v>
       </c>
       <c r="K16" s="10"/>
     </row>
     <row r="17">
-      <c r="B17" s="13">
+      <c r="B17" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="14">
         <v>46327.0</v>
       </c>
       <c r="D17" s="8">
         <v>14.9</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="15">
         <f t="shared" si="2"/>
         <v>16.9115</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="20">
         <v>128394.0</v>
       </c>
       <c r="K17" s="1"/>
     </row>
     <row r="18">
-      <c r="B18" s="13">
+      <c r="B18" s="14">
         <v>46314.0</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="14">
         <v>46327.0</v>
       </c>
       <c r="D18" s="8">
         <v>12.5</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="15">
         <f t="shared" si="2"/>
         <v>14.1875</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="17" t="s">
         <v>38</v>
       </c>
       <c r="I18" s="9">

</xml_diff>

<commit_message>
Add week 45-46 offer pages and Instagram images
Build both offer pages and the 12 product Instagram images from the
week 45-46 spreadsheet, photos and recipe QR codes, with photo
adjustments to keep products clear of price badges. Move the week
43-44 spreadsheet and QR codes to arkisto/vko-43-44.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8Lk915b9RmWmbPNMZUzmb
</commit_message>
<xml_diff>
--- a/viikkotarjoukset/tarjoukset.xlsx
+++ b/viikkotarjoukset/tarjoukset.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
   <si>
     <t>Page 1</t>
   </si>
@@ -50,49 +50,49 @@
     <t>kg</t>
   </si>
   <si>
-    <t>Hätälä lohimurekemassa</t>
+    <t>Atria takuumurea naudan sisäpaisti</t>
   </si>
   <si>
-    <t>Pakaste, Suomi, n.6,6kg/ltk</t>
+    <t>Tuore, Suomi, n.5,5kg/kpl</t>
   </si>
   <si>
-    <t>Lohiwallenberg, perunamuusi ja pikkelöidyt kasvikset rapukastikkeella</t>
+    <t>Naudanliha-kaalipata ja puolukkaa</t>
   </si>
   <si>
-    <t>Miyata pankojauho</t>
+    <t>Arla Keittiö laktoositon smetana</t>
   </si>
   <si>
-    <t>Kiina, 10x1kg/me</t>
+    <t>Tuore, Suomi, 1,8kg/kpl</t>
   </si>
   <si>
-    <t>Atria possun tryffelikassler</t>
+    <t>Atria kanan miedosti suolattu filee n.150g</t>
   </si>
   <si>
-    <t>Tuore, Suomi, n.2,8kg/kpl</t>
+    <t>Tuore, Suomi, n.3kg/kpl</t>
   </si>
   <si>
-    <t>Tryffelipossua ja karamellisipulikastiketta</t>
+    <t>Valkosipuli-timjamivoissa paistettua kanaa</t>
   </si>
   <si>
-    <t>Atria sydänmerkki perunasose</t>
+    <t>Atria Säräjuuresainekset</t>
   </si>
   <si>
-    <t>Tuore, Suomi, 4kg/kpl</t>
+    <t>Tuore, Suomi, 2,5kg/kpl</t>
   </si>
   <si>
-    <t>Lagerblad Foods lammaspyörykkä 16g</t>
+    <t>Saarioinen täytetty kievin broileripyörykkä</t>
   </si>
   <si>
-    <t>Pakaste, Suomi, 6kg/ltk</t>
+    <t>Pakaste, Suomi, 4kg/ltk</t>
   </si>
   <si>
-    <t>Shepherds pie lammaspyöryköistä</t>
+    <t>Kievin kanapyöryköitä, currykastiketta ja mausteista omenaa</t>
   </si>
   <si>
-    <t>Patu tomaattimurska</t>
+    <t>Saarioinen Currykastike</t>
   </si>
   <si>
-    <t>EU, 12x1kg/me</t>
+    <t>Suomi, 2kg/kpl</t>
   </si>
   <si>
     <t>Page 2</t>
@@ -101,40 +101,46 @@
     <t>Partner</t>
   </si>
   <si>
-    <t>Pangasiusfilee 120-170g</t>
+    <t>PNM</t>
   </si>
   <si>
-    <t>Pakaste, Vietnam, 10kg/ltk</t>
+    <t>Atria viljaporsaan kasleri</t>
   </si>
   <si>
-    <t>Merhav Hoki Annospala Luomupaneroitu 50g</t>
+    <t>Tuore, Suomi, n.2,5kg/kpl</t>
   </si>
   <si>
-    <t>Pakaste, Ruotsi, 5kg/ltk</t>
+    <t>Kalaneuvos tuore kirjolohifilee c-leikkuu</t>
   </si>
   <si>
-    <t>Familia Pro Porsaan kypsä ulkofileeleike 120g</t>
-  </si>
-  <si>
-    <t>Pakaste, Saksa, 7,2kg/ltk</t>
-  </si>
-  <si>
-    <t>HK Uunimakkara 80g</t>
+    <t>Tuore, Suomi, n.5kg/ltk</t>
   </si>
   <si>
     <t>kpl</t>
   </si>
   <si>
-    <t>Eesti Pagar laktoositon porkkanakakku, 32 palaa</t>
+    <t>Eesti pagar Appelsiini-suklaakakku, 10 palaa</t>
   </si>
   <si>
-    <t>Pakaste, Viro, 3x1,8kg/me</t>
+    <t>Pakaste, Viro, 4x950g/ltk</t>
   </si>
   <si>
-    <t>Sauvon maustekurkkukuutio</t>
+    <t>Lagerblad foods gluteeniton jättilihapulla</t>
   </si>
   <si>
-    <t>Suomi, 8,2kg/4.3kg</t>
+    <t>Pakaste, Suomi, 5kg/ltk</t>
+  </si>
+  <si>
+    <t>HK uunimakkara 50x80g</t>
+  </si>
+  <si>
+    <t>Tuore, Suomi, 4kg/kpl</t>
+  </si>
+  <si>
+    <t>Saarioinen kermaperunat</t>
+  </si>
+  <si>
+    <t>Tuore, Suomi, 2,6kg/kpl</t>
   </si>
 </sst>
 </file>
@@ -144,7 +150,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -179,22 +185,28 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <sz val="39.0"/>
+      <color rgb="FF0B6E41"/>
+      <name val="Sini-500"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <sz val="29.0"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
     </font>
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="54.0"/>
+      <color rgb="FFDC241F"/>
+      <name val="Lora"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -203,21 +215,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCE6F1"/>
-        <bgColor rgb="FFDCE6F1"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF6E9"/>
+        <bgColor rgb="FFFFF6E9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <top style="thin">
-        <color rgb="FF95B3D7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF95B3D7"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
@@ -251,20 +261,20 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="2" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -276,8 +286,8 @@
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,17 +562,17 @@
     </row>
     <row r="3">
       <c r="B3" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C3" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D3" s="4">
-        <v>7.9</v>
+        <v>16.6</v>
       </c>
       <c r="E3" s="2">
         <f t="shared" ref="E3:E8" si="1">D3*1.135</f>
-        <v>8.9665</v>
+        <v>18.841</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>9</v>
@@ -574,25 +584,26 @@
         <v>11</v>
       </c>
       <c r="I3" s="6">
-        <v>137653.0</v>
+        <v>111265.0</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>12</v>
       </c>
+      <c r="M3" s="7"/>
     </row>
     <row r="4">
       <c r="B4" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C4" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D4" s="8">
-        <v>4.4</v>
+        <v>7.17</v>
       </c>
       <c r="E4" s="2">
         <f t="shared" si="1"/>
-        <v>4.994</v>
+        <v>8.13795</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>9</v>
@@ -604,7 +615,7 @@
         <v>14</v>
       </c>
       <c r="I4" s="6">
-        <v>145141.0</v>
+        <v>104826.0</v>
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="7" t="s">
@@ -613,29 +624,29 @@
     </row>
     <row r="5">
       <c r="B5" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C5" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D5" s="4">
-        <v>8.9</v>
+        <v>7.99</v>
       </c>
       <c r="E5" s="2">
         <f t="shared" si="1"/>
-        <v>10.1015</v>
+        <v>9.06865</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="6">
-        <v>131717.0</v>
+        <v>100186.0</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>17</v>
@@ -643,17 +654,17 @@
     </row>
     <row r="6">
       <c r="B6" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C6" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D6" s="4">
-        <v>4.73</v>
+        <v>7.2</v>
       </c>
       <c r="E6" s="2">
         <f t="shared" si="1"/>
-        <v>5.36855</v>
+        <v>8.172</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>9</v>
@@ -665,7 +676,7 @@
         <v>19</v>
       </c>
       <c r="I6" s="7">
-        <v>138990.0</v>
+        <v>130338.0</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>17</v>
@@ -674,48 +685,49 @@
     <row r="7">
       <c r="A7" s="1"/>
       <c r="B7" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C7" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D7" s="4">
-        <v>11.99</v>
+        <v>8.99</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="1"/>
-        <v>13.60865</v>
+        <v>10.20365</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>21</v>
       </c>
       <c r="I7" s="7">
-        <v>110285.0</v>
+        <v>144684.0</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="T7" s="11"/>
     </row>
     <row r="8">
       <c r="A8" s="1"/>
       <c r="B8" s="3">
-        <v>46314.0</v>
+        <v>46328.0</v>
       </c>
       <c r="C8" s="3">
-        <v>46327.0</v>
+        <v>46341.0</v>
       </c>
       <c r="D8" s="4">
-        <v>1.99</v>
+        <v>5.6</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="1"/>
-        <v>2.25865</v>
+        <v>6.356</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>9</v>
@@ -727,18 +739,21 @@
         <v>24</v>
       </c>
       <c r="I8" s="7">
-        <v>142394.0</v>
+        <v>144753.0</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="L8" s="12"/>
+      <c r="T8" s="13"/>
     </row>
     <row r="9">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="13"/>
+      <c r="C9" s="14"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
+      <c r="L9" s="15"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
@@ -747,7 +762,9 @@
       <c r="B10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="13"/>
+      <c r="C10" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
@@ -781,170 +798,170 @@
       <c r="K12" s="1"/>
     </row>
     <row r="13">
-      <c r="B13" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C13" s="14">
-        <v>46327.0</v>
+      <c r="B13" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>46341.0</v>
       </c>
       <c r="D13" s="8">
-        <v>5.1</v>
-      </c>
-      <c r="E13" s="15">
+        <v>5.9</v>
+      </c>
+      <c r="E13" s="16">
         <f t="shared" ref="E13:E18" si="2">D13*1.135</f>
-        <v>5.7885</v>
-      </c>
-      <c r="F13" s="16" t="s">
+        <v>6.6965</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I13" s="18">
-        <v>133952.0</v>
+        <v>100257.0</v>
       </c>
       <c r="K13" s="19"/>
     </row>
     <row r="14">
-      <c r="B14" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C14" s="14">
-        <v>46327.0</v>
+      <c r="B14" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>46341.0</v>
       </c>
       <c r="D14" s="8">
-        <v>6.8</v>
-      </c>
-      <c r="E14" s="15">
+        <v>12.0</v>
+      </c>
+      <c r="E14" s="16">
         <f t="shared" si="2"/>
-        <v>7.718</v>
-      </c>
-      <c r="F14" s="16" t="s">
+        <v>13.62</v>
+      </c>
+      <c r="F14" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" s="16" t="s">
+      <c r="G14" s="17" t="s">
         <v>30</v>
       </c>
+      <c r="H14" s="17" t="s">
+        <v>31</v>
+      </c>
       <c r="I14" s="18">
-        <v>143955.0</v>
+        <v>140241.0</v>
       </c>
       <c r="K14" s="19"/>
     </row>
     <row r="15">
-      <c r="B15" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C15" s="14">
-        <v>46327.0</v>
+      <c r="B15" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>46341.0</v>
       </c>
       <c r="D15" s="8">
-        <v>8.62</v>
-      </c>
-      <c r="E15" s="15">
+        <v>13.9</v>
+      </c>
+      <c r="E15" s="16">
         <f t="shared" si="2"/>
-        <v>9.7837</v>
-      </c>
-      <c r="F15" s="16" t="s">
+        <v>15.7765</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="18">
+        <v>144153.0</v>
+      </c>
+      <c r="K15" s="10"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>46341.0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>9.8</v>
+      </c>
+      <c r="E16" s="16">
+        <f t="shared" si="2"/>
+        <v>11.123</v>
+      </c>
+      <c r="F16" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="I15" s="18">
-        <v>129487.0</v>
-      </c>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C16" s="14">
-        <v>46327.0</v>
-      </c>
-      <c r="D16" s="8">
-        <v>4.75</v>
-      </c>
-      <c r="E16" s="15">
+      <c r="G16" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="18">
+        <v>114377.0</v>
+      </c>
+      <c r="K16" s="10"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>46341.0</v>
+      </c>
+      <c r="D17" s="8">
+        <v>4.38</v>
+      </c>
+      <c r="E17" s="16">
         <f t="shared" si="2"/>
-        <v>5.39125</v>
-      </c>
-      <c r="F16" s="16" t="s">
+        <v>4.9713</v>
+      </c>
+      <c r="F17" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="I16" s="18">
+      <c r="G17" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="I17" s="20">
         <v>103157.0</v>
       </c>
-      <c r="K16" s="10"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C17" s="14">
-        <v>46327.0</v>
-      </c>
-      <c r="D17" s="8">
-        <v>14.9</v>
-      </c>
-      <c r="E17" s="15">
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="3">
+        <v>46328.0</v>
+      </c>
+      <c r="C18" s="3">
+        <v>46341.0</v>
+      </c>
+      <c r="D18" s="8">
+        <v>3.85</v>
+      </c>
+      <c r="E18" s="16">
         <f t="shared" si="2"/>
-        <v>16.9115</v>
-      </c>
-      <c r="F17" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="H17" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="20">
-        <v>128394.0</v>
-      </c>
-      <c r="K17" s="1"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="14">
-        <v>46314.0</v>
-      </c>
-      <c r="C18" s="14">
-        <v>46327.0</v>
-      </c>
-      <c r="D18" s="8">
-        <v>12.5</v>
-      </c>
-      <c r="E18" s="15">
-        <f t="shared" si="2"/>
-        <v>14.1875</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" s="21" t="s">
-        <v>37</v>
+        <v>4.36975</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>39</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I18" s="9">
-        <v>103821.0</v>
+        <v>111201.0</v>
       </c>
     </row>
     <row r="19">
@@ -978,6 +995,7 @@
     <row r="26" ht="15.75" customHeight="1">
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
+      <c r="P26" s="21"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="D27" s="2"/>

</xml_diff>

<commit_message>
Apply week 45-46 spreadsheet corrections
Add product weights to the kievin broileripyörykkä and jättilihapulla
names and fix the Eesti Pagar and Lagerblad Foods capitalisation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8Lk915b9RmWmbPNMZUzmb
</commit_message>
<xml_diff>
--- a/viikkotarjoukset/tarjoukset.xlsx
+++ b/viikkotarjoukset/tarjoukset.xlsx
@@ -80,7 +80,7 @@
     <t>Tuore, Suomi, 2,5kg/kpl</t>
   </si>
   <si>
-    <t>Saarioinen täytetty kievin broileripyörykkä</t>
+    <t>Saarioinen täytetty kievin broileripyörykkä 20g</t>
   </si>
   <si>
     <t>Pakaste, Suomi, 4kg/ltk</t>
@@ -119,13 +119,13 @@
     <t>kpl</t>
   </si>
   <si>
-    <t>Eesti pagar Appelsiini-suklaakakku, 10 palaa</t>
+    <t>Eesti Pagar Appelsiini-suklaakakku, 10 palaa</t>
   </si>
   <si>
     <t>Pakaste, Viro, 4x950g/ltk</t>
   </si>
   <si>
-    <t>Lagerblad foods gluteeniton jättilihapulla</t>
+    <t>Lagerblad Foods gluteeniton jättilihapulla 50g</t>
   </si>
   <si>
     <t>Pakaste, Suomi, 5kg/ltk</t>
@@ -150,7 +150,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -200,6 +200,11 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b/>
       <sz val="54.0"/>
       <color rgb="FFDC241F"/>
@@ -232,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -260,6 +265,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -283,10 +291,13 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -700,7 +711,7 @@
       <c r="F7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="11" t="s">
         <v>20</v>
       </c>
       <c r="H7" s="9" t="s">
@@ -712,7 +723,7 @@
       <c r="K7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="T7" s="11"/>
+      <c r="T7" s="12"/>
     </row>
     <row r="8">
       <c r="A8" s="1"/>
@@ -744,16 +755,16 @@
       <c r="K8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="T8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="T8" s="14"/>
     </row>
     <row r="9">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="14"/>
+      <c r="C9" s="15"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="L9" s="15"/>
+      <c r="L9" s="16"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
@@ -807,23 +818,23 @@
       <c r="D13" s="8">
         <v>5.9</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="17">
         <f t="shared" ref="E13:E18" si="2">D13*1.135</f>
         <v>6.6965</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="18" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="19">
         <v>100257.0</v>
       </c>
-      <c r="K13" s="19"/>
+      <c r="K13" s="20"/>
     </row>
     <row r="14">
       <c r="B14" s="3">
@@ -835,23 +846,23 @@
       <c r="D14" s="8">
         <v>12.0</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="17">
         <f t="shared" si="2"/>
         <v>13.62</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="19">
         <v>140241.0</v>
       </c>
-      <c r="K14" s="19"/>
+      <c r="K14" s="20"/>
     </row>
     <row r="15">
       <c r="B15" s="3">
@@ -863,20 +874,20 @@
       <c r="D15" s="8">
         <v>13.9</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="17">
         <f t="shared" si="2"/>
         <v>15.7765</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="H15" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="19">
         <v>144153.0</v>
       </c>
       <c r="K15" s="10"/>
@@ -891,20 +902,20 @@
       <c r="D16" s="8">
         <v>9.8</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="17">
         <f t="shared" si="2"/>
         <v>11.123</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="H16" s="17" t="s">
+      <c r="H16" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="19">
         <v>114377.0</v>
       </c>
       <c r="K16" s="10"/>
@@ -919,20 +930,20 @@
       <c r="D17" s="8">
         <v>4.38</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="17">
         <f t="shared" si="2"/>
         <v>4.9713</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="18" t="s">
         <v>9</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="22">
         <v>103157.0</v>
       </c>
       <c r="K17" s="1"/>
@@ -947,17 +958,17 @@
       <c r="D18" s="8">
         <v>3.85</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="17">
         <f t="shared" si="2"/>
         <v>4.36975</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="18" t="s">
         <v>9</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H18" s="18" t="s">
         <v>40</v>
       </c>
       <c r="I18" s="9">
@@ -995,7 +1006,7 @@
     <row r="26" ht="15.75" customHeight="1">
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
-      <c r="P26" s="21"/>
+      <c r="P26" s="23"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="D27" s="2"/>

</xml_diff>